<commit_message>
Organise study-level download list into batches after completeness re-check
Re-checked Unclear records, DIRECT/NRSI exclusions and all ANCHORED abstracts;
added the resulting candidates (Batch 5 and registry checks) and a batch
checklist with per-batch workbook sheets for full-text decisions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FZknuUfJxYKgLwkTzEMVHD
</commit_message>
<xml_diff>
--- a/study_selection/Study_Selection.xlsx
+++ b/study_selection/Study_Selection.xlsx
@@ -7,9 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Download_List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Record_Map_312" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reference_MAs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BATCH_1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BATCH_2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BATCH_3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BATCH_4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BATCH_5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Download_List" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Record_Map_312" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Reference_MAs" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,13 +434,3159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Download?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main record (Screen_ID)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Link (main record)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Title (main record)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Companion records (merge, do not count)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / what to check at full text</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Downloaded? (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Full-text decision</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reason if excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dickson 1991</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam 0.5% gel vs oral ibuprofen 400 mg tid</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S13654</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=A%20double-blind%20evaluation%20of%20topical%20piroxicam%20gel%20with%20oral%20ibuprofen%20in%20osteoarthritis%20of%20the%20knee</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>A double-blind evaluation of topical piroxicam gel with oral ibuprofen in osteoarthritis of the knee</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>CSV sample_n=118 is one arm only; abstract states 235 randomised.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Sandelin 1997</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Eltenac gel vs oral diclofenac vs placebo gel</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>290</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S14932</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/9310109/</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Local NSAID gel (Eltenac) in the treatment of osteoarthritis of the knee: A double blind study comparing eltenac with oral diclofenac and placebo gel</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Has placebo arm (anchors network).</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tugwell 2004</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac 1.5% in DMSO (Pennsaid) vs oral diclofenac</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S21608</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/15468367/</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Equivalence study of a topical diclofenac solution (pennsaid) compared with oral diclofenac in symptomatic treatment of osteoarthritis of the knee: a randomized controlled trial.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>S20740 (2003 ARD abstract)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Rother 2007</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Ketoprofen in Transfersome (IDEA-033) vs oral celecoxib vs placebo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>397</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S19119</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/17363401/</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and safety of epicutaneous ketoprofen in transfersome (IDEA-033) versus oral celecoxib and placebo in osteoarthritis of the knee: Multicentre randomised controlled trial</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>possibly S16986 (NCT00317733) - confirm</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Has placebo arm.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Simon 2009</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac/DMSO vs DMSO vehicle vs placebo vs oral diclofenac vs TOPICAL+ORAL</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>775</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S13265</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/19380203/</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and safety of topical diclofenac containing dimethyl sulfoxide (DMSO) compared with those of topical placebo, DMSO vehicle and oral diclofenac for knee osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>S23676 (2008 abstract); probably S16905 (NCT00108992)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>KEY trial: only double-blind trial with a topical+oral arm - connects the combination node to both topical and oral.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Doi 2010</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>NSAID plasters vs oral NSAIDs (top-3 Japanese products in each arm)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>165 analysed</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S10579</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/19806426/</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Effect of nonsteroidal anti-inflammatory drug plasters for knee osteoarthritis in Japanese: A randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Class-level comparison (several products per arm); open-label -&gt; RoB.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tiso 2010</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Oral ibuprofen vs topical 4% ibuprofen gel</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>20 (per CSV)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>S04144</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/20859315/</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Oral versus topical ibuprofen for chronic knee pain: A prospective randomized pilot study</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Very small pilot.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Conaghan 2013</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>IDEA-033 ketoprofen (50/100 mg) vs TDT064 vehicle vs oral celecoxib 100 mg bid vs oral placebo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1395</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>S20992</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/23542612/</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>A multicentre, randomized, placebo- and active-controlled trial comparing the efficacy and safety of topical ketoprofen in Transfersome gel (IDEA-033) with ketoprofen-free vehicle (TDT 064) and oral celecoxib for knee pain associated with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>S21659 (EULAR 2013 abstract); S13479 (NCT00716547)</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Largest trial. Has placebo arms.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Mu 2016</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Loxoprofen hydrogel patch vs loxoprofen tablet</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>169 (per 2013 abstract)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>S18896</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/24924603/</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and safety of loxoprofen hydrogel patch versus loxoprofen tablet in patients with knee osteoarthritis: a randomized controlled non-inferiority trial</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>S10033 (2013 IJRD abstract)</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Shinde 2017</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>YES (conditional)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Transdermal diclofenac patch vs oral diclofenac SR</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>S13012</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29472748/</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and safety of oral diclofenac sustained release versus transdermal diclofenac patch in chronic musculoskeletal pain: A randomized, open label trial</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Keep only if knee-OA results are reported separately; otherwise exclude (wrong population). Zeng 2021 did not include it.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Download?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main record (Screen_ID)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Link (main record)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Title (main record)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Companion records (merge, do not count)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / what to check at full text</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Downloaded? (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Full-text decision</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reason if excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Underwood 2008 (TOIB)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Advice to use topical vs oral ibuprofen</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>282 in RCT arm</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S14978 (HTA full report)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/18505668/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Topical or oral ibuprofen for chronic knee pain in older people. The TOIB study</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>S17792 (BMJ 2008 main paper - download too); S01645 (cost-effectiveness); S23429 (protocol)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Use RCT arm only. Advice-based intervention and knee-pain population differ from other trials: sensitivity analysis without it.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Rother, Yeoman &amp; Ekman 2013</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>YES (look for full paper)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>IDEA-033 ketoprofen 25/50/100 mg vs oral naproxen vs placebo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>837</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S15749 (EULAR 2013 abstract)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/annrheumdis-2012-eular.3275</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>A double-blind, placebo-controlled trial comparing the safety and efficacy of epicutaneously applied ketoprofen in transfersome gel with naproxen for the treatment of pain associated with osteoarthritis (OA) of the knee</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>S10501 (NCT00211549)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2nd-largest trial. I could not check whether a full paper exists (PubMed tool failed). Check ClinicalTrials.gov NCT00211549 for posted results. If only an abstract exists, follow your protocol rule on abstracts; run a sensitivity analysis without it.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Takagishi 1985 (MEN-OM)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Ketoprofen 3% ointment vs oral ketoprofen 50 mg tid</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S18409</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Evaluation%20of%20MEN-OM%20in%20the%20Treatment%20of%20Osteoarthritis%20of%20the%20Knee%20-A%20Double-Blind%20Comparative%20Study-</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Evaluation of MEN-OM in the Treatment of Osteoarthritis of the Knee -A Double-Blind Comparative Study-</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Authors call the oral arm an "active placebo" but it is full-dose oral ketoprofen: a genuine topical-vs-oral comparison.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Tsuyama 1985 (L-141)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>L-141 NSAID ointment vs "FB" tablet (oral NSAID; confirm drug)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>275</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S15553</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Evaluation%20of%20L-141%20Ointment%20on%20Arthritis%20Deformans%20of%20Knee</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Evaluation of L-141 Ointment on Arthritis Deformans of Knee</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Confirm what the L-141 and FB drugs are.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ozgen 2011</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac epolamine plaster (Flector) vs oral diclofenac SR vs no treatment</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S12474</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Efficiency%20of%20local%20diclophenac%20treatment%20in%20knee%20osteoartritis</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Efficiency of local diclophenac treatment in knee osteoartritis</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Very small.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Liu 2025</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Oral loxoprofen vs flurbiprofen gel patch vs ORAL+TOPICAL</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S18337</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=%E5%8F%A3%E6%9C%8D%E6%B4%9B%E7%B4%A2%E6%B4%9B%E8%8A%AC%E9%92%A0%E7%89%87%E8%81%94%E5%90%88%E6%B0%9F%E6%AF%94%E6%B4%9B%E8%8A%AC%E5%87%9D%E8%83%B6%E8%B4%B4%E8%86%8F%E6%B2%BB%E7%96%97%E8%86%9D%E9%AA%A8%E5%85%B3%E8%8A%82%E7%82%8E%E7%9A%84%E4%B8%B4%E5%BA%8A%E7%96%97%E6%95%88%E4%B8%8E%E5%AE%89%E5%85%A8%E6%80%A7%E7%A0%94%E7%A9%B6</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>口服洛索洛芬钠片联合氟比洛芬凝胶贴膏治疗膝骨关节炎的临床疗效与安全性研究</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Also feeds the combination node (closed topical-oral-combination loop).</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Kageyama 1986 (KPG-200)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>YES (if retrievable)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Ketoprofen ointment vs oral ketoprofen</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>S11142</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Efficacy%20of%20KPG-200%20%28Ketoprofen%20Ointment%29%20to%20Gonarthrosis%3A%20double-Blind%20Controlled%20Trials%20Using%20Oral%20Ketoprofen%20as%20Control</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Efficacy of KPG-200 (Ketoprofen Ointment) to Gonarthrosis: double-Blind Controlled Trials Using Oral Ketoprofen as Control</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>No abstract: confirm randomisation and data.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Nagaya 1984</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>YES (if retrievable)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam gel vs piroxicam capsule</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>S07754</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=A%20Double%20Blind%20Comparative%20Study%20of%20Piroxicam%20Gel%20and%20Piroxicam%20Capsule%20in%20the%20Treatment%20of%20Osteoarthritis</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>A Double Blind Comparative Study of Piroxicam Gel and Piroxicam Capsule in the Treatment of Osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>No abstract: confirm knee OA, randomisation and data.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Download?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main record (Screen_ID)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Link (main record)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Title (main record)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Companion records (merge, do not count)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / what to check at full text</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Downloaded? (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Full-text decision</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reason if excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Sun 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Oral celecoxib 200 mg qd + flurbiprofen patch bid vs celecoxib alone</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S03016</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/42714961/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Celecoxib plus topical flurbiprofen patch versus celecoxib alone for symptomatic knee OA: a randomized controlled trial.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Wang 2023</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Oral celecoxib 100 mg bid + diclofenac cream tid vs celecoxib alone</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S25587</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.13699/j.cnki.1001-6821.2023.15.009</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>塞来昔布联合双氯芬酸钠治疗膝关节骨关节炎患者的临床研究</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Zhang 2011</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Oral diclofenac 25 mg tid + diclofenac gel vs oral diclofenac alone</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S19208</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=%E5%A4%9A%E6%A8%A1%E5%BC%8F%E9%95%87%E7%97%9B%E6%B2%BB%E7%96%97%E8%80%81%E5%B9%B4%E8%86%9D%E5%85%B3%E8%8A%82%E9%AA%A8%E5%85%B3%E8%8A%82%E7%82%8E%E7%9A%84%E4%B8%B4%E5%BA%8A%E7%A0%94%E7%A9%B6</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>多模式镇痛治疗老年膝关节骨关节炎的临床研究</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Dehghan 2019 (Thymus gel)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac 1% gel + oral celecoxib vs placebo gel + oral celecoxib (3rd arm: herbal gel - ignore)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S05874</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31124455/</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Comparative study of the effect of Thymus daenensis gel 5% and diclofenac in patients with knee osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>MISFILED as ANCHORED: every arm took oral celecoxib, so diclofenac gel vs placebo gel = combination vs oral alone.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Dehghan 2018 (ginger jelly)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam jelly + oral diclofenac 100 mg/d vs placebo jelly + oral diclofenac (3rd arm: herbal - ignore)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>English abstract</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S04875</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Comparison%20the%20effects%20of%20ginger%20%28Zingiber%20officinale%29%20jelly%20and%20piroxicam%20jelly%20on%20pain%20of%20knee%20osteoarthritis</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Comparison the effects of ginger (Zingiber officinale) jelly and piroxicam jelly on pain of knee osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>MISFILED as ANCHORED (same logic as above). Check that allocation was truly randomised.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Sasaki 2021</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>YES (verify design)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>S-flurbiprofen plaster alone vs conventional oral + topical NSAIDs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S16015</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34316523/</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Treatment Efficacy of Single Topical NSAID (S-Flurbiprofen Plaster) for Knee Symptoms and Locomotive Dysfunction in Knee Osteoarthritis Patients.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>possibly S24573 (jRCTs021180050 NEXT study) - confirm</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Topical-vs-combination edge. If not randomised, move to NRSI or exclude.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Download?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main record (Screen_ID)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Link (main record)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Title (main record)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Companion records (merge, do not count)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / what to check at full text</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Downloaded? (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Full-text decision</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reason if excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Zeng 2021 THIN cohort</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>YES (you already have the PDF)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Topical vs oral NSAID initiators</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>14,218 per group</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S24435</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34174454/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Comparative efficacy and safety of acetaminophen, topical and oral non-steroidal anti-inflammatory drugs for knee osteoarthritis: evidence from a network meta-analysis of randomized controlled trials and real-world data</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>ADD: currently excluded as REVIEW-LIST, but the paper contains original knee-OA cohort data (mortality, CVD, VTE, GI bleeding). The most relevant NRSI you have.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Silverman 2022</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Oral tNSAIDs vs topical NSAIDs vs COX-2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S25286</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/35575236/</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Drug utilization, clinical and economic outcomes of patients with osteoarthritis of the hip and/or knee treated with long-term use of traditional NSAIDs, topical NSAIDs, and COX-2 inhibitors</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>S06033 (EULAR 2021 abstract)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Check if knee-only data are separable.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Keshwani 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Topical vs oral NSAID initiation</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S24685</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/41833532/</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Association Between Different Analgesic Use and Hypertension Among Medicare Beneficiaries With Osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Outcome: hypertension.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Pontes 2018</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Topical NSAIDs vs oral NSAIDs (exposure categories)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S12226</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29398161/</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Analgesic Use and Risk for Acute Coronary Events in Patients With Osteoarthritis: A Population-based, Nested Case-control Study</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Outcome: acute coronary events.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Kikuchi 2021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>YES (verify)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Oral vs topical NSAID users</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S07334 (Unclear at T/A)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/33585939/</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>A Retrospective Database Study of Gastrointestinal Events and Medical Costs Associated with Nonsteroidal Anti-Inflammatory Drugs in Japanese Patients of Working Age with Osteoarthritis and Chronic Low Back Pain</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>GI events and costs. PMID 33585939.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Schoffski 2000</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>YES (low priority)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac (Emulgel) vs oral NSAIDs vs both</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1525</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S25055</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1055/s-2008-1043511</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac (Emulgel) vs. oral NSAIDs in therapy of gonarthrosis and fingerarthrosis - A cost analysis</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Keep only if it reports adverse-event outcomes (mainly a cost study).</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sinnott 2020</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Oral NSAIDs vs topical diclofenac</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>see full text</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>S05175</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pds.5114</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Evaluating signals generated in a large-scale sequence symmetry analysis: Macrolides and heart failure; NSAIDs and pneumonia</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Outcome is pneumonia; include only if pneumonia is a protocol safety outcome.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Study</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Download?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main record (Screen_ID)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Link (main record)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Title (main record)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Companion records (merge, do not count)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / what to check at full text</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Downloaded? (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Full-text decision</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Reason if excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Koyama 2022 (OASIS DUAL)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Duloxetine + S-flurbiprofen plaster vs duloxetine + oral NSAIDs</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S20814</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/36223938/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Comparison of efficacy and safety in the combination therapies of duloxetine and S-flurbiprofen plaster, and of duloxetine and conventional NSAIDs for chronic pain in patients with osteoarthritis (OASIS DUAL study).</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Randomisation not reported; n=49; 9-mo follow-up. Likely non-randomised -&gt; exclude or NRSI.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Hashimoto 2018</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>HA injection + S-flurbiprofen plaster vs HA + oral NSAID vs HA alone</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S00867</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Combination%20therapy%20of%20intra-articular%20hyaluronan%20injection%20and%20S-flurbiprofen%20plaster%20for%20knee%20osteoarthritis</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Combination therapy of intra-articular hyaluronan injection and S-flurbiprofen plaster for knee osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>"Divided into three groups": randomisation not stated.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Aoki 1990 (SR-318)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>SR-318 vs diclofenac tablets, double-blind, knee OA</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S05437</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Evaluation%20of%20SR-318%20on%20Osteoarthritis%20of%20Knee%20Joint%3A%20double%20Blind%20Comparative%20Study%20with%20Diclofenac%20Sodium%20Tablets</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Evaluation of SR-318 on Osteoarthritis of Knee Joint: double Blind Comparative Study with Diclofenac Sodium Tablets</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A: is SR-318 topical? If yes -&gt; P2.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Miura 1987 (HKP-210)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>HKP-210 vs oral ketoprofen, double-blind, knee OA</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S07052</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Evaluation%20of%20HKP-210%20in%20Osteoarthritis%20of%20the%20Knee%3A%20a%20Double-Blind%20Comparison%20with%20Oral%20Ketoprofen</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Evaluation of HKP-210 in Osteoarthritis of the Knee: a Double-Blind Comparison with Oral Ketoprofen</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A: is HKP-210 topical? If yes -&gt; P2.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Browning 1994</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Reduced oral NSAID + piroxicam gel vs usual oral NSAID, elderly OA</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S13555</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/10150264/</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Reducing the dose of oral NSAIDs by use of Feldene Gel: An open study in elderly patients with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Open study; randomisation and knee unclear. PMID 10150264.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Rau 1992</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam ointment added to systemic therapy, activated gonarthrosis</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>S24647</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Therapy%20of%20activated%20gonarthrosis%20with%20piroxicam%20ointment%3A%20Significant%20completion%20of%20systemic%20therapy</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Therapy of activated gonarthrosis with piroxicam ointment: Significant completion of systemic therapy</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>No abstract; possible combination design.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Blumberger 1980</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Etofenamate gel to reduce oral antirheumatic dose</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>S16115</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Reduction%20of%20required%20dosage%20of%20antirheumatic%20agents%20by%20local%20use%20of%20etofenamate%20gel</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Reduction of required dosage of antirheumatic agents by local use of etofenamate gel</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>No abstract; possible combination design.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Aoki 1992 (BPAA)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BPAA vs indomethacin patch</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>S05399</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20Evaluation%20of%20BPAA%20on%20Osteoarthritis%20of%20the%20Knee%3A%20a%20Multicenter%20Comparative%20Study%20with%20Indomethacin%20Patch</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Evaluation of BPAA on Osteoarthritis of the Knee: a Multicenter Comparative Study with Indomethacin Patch</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Probably topical vs topical -&gt; likely exclude.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Kurata 1997 (FO-726)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>FO-726 vs indomethacin cataplasm</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>S09693</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20evaluation%20of%20FO-726%20in%20osteoarthrosis%3A%20Clinical%20comparative%20study%20versus%20commercially%20available%20indomethacin%20cataplasm</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Clinical evaluation of FO-726 in osteoarthrosis: Clinical comparative study versus commercially available indomethacin cataplasm</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Probably topical vs topical -&gt; likely exclude.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Bolten 1994</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Flurbiprofen LAT vs oral flurbiprofen/ibuprofen</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>S22478</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/7917798/</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>The pharmacokinetics, pharmacodynamics and comparative efficacy of flurbiprofen lat</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Probably a narrative summary -&gt; likely exclude.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Roth 1995 (diclofenac/hyaluronan gel)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac 3%/hyaluronan gel vs placebo gel in patients with uncontrolled pain on CHRONIC ORAL NSAIDs</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>S00576</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/8867642/</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>A controlled clinical investigation of 3% diclofenac/2.5% sodium hyaluronate topical gel in the treatment of uncontrolled pain in chronic oral NSAID users with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>S14701 (RSM Round Table report)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Was Unclear/ANCHORED. If patients kept taking their oral NSAID and it is knee OA, this is topical+oral vs oral -&gt; combination node.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Togo 2022</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Oral vs non-oral NSAID users (main comparison is age &gt;=65 vs &lt;65)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>288,715</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>S20244</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34538031/</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Safety risk associated with use of nonsteroidal anti-inflammatory drugs in Japanese elderly compared with younger patients with osteoarthritis and/or chronic low back pain: A retrospective database study</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>WRONGLY REASONED EXCLUSION at T/A ("no placebo" does not apply to cohorts). Same database/group as Kikuchi 2021. Include only if it reports outcomes by route in OA patients. PMID 34538031.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac potassium 1% gel (2002, Chinese)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac potassium gel; comparator unknown (abstract = keywords only)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>S01109</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Effect%20and%20safety%20of%201%25%20diclofenac%20potassium%20gel%20for%20external%20application%20in%20treatment%20of%20patients%20with%20osteoarthritis</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Effect and safety of 1% diclofenac potassium gel for external application in treatment of patients with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Transdermal diclofenac multicentre trial (1987)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Transdermal diclofenac; comparator unknown</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>S21573</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Transdermic%20application%20of%20diclofenac%20-%20Results%20of%20a%20multicenter%20trial</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Transdermic application of diclofenac - Results of a multicenter trial</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam gel in gonarthrosis (1993)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Topical piroxicam gel; comparator unknown</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>S22576</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Efficacy%20and%20tolerance%20of%20piroxicam%20gel.%20Percutaneous%20nonsteroidal%20antirheumatic%20agents%20in%20the%20treatment%20of%20gonarthrosis</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and tolerance of piroxicam gel. Percutaneous nonsteroidal antirheumatic agents in the treatment of gonarthrosis</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Ketorolac gel 1% long-term (1993)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Topical ketorolac, knee OA; comparator unknown</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>S10571</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Long-term%20efficacy%20of%20ketorolac%20Gel%201%25%20in%20patients%20suffering%20from%20osteoarthritis%20of%20the%20knee</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Long-term efficacy of ketorolac Gel 1% in patients suffering from osteoarthritis of the knee</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Diclo Duo spray (2010)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac spray; comparator unknown</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>S05441</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/21875024/</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>[Topical treatment with diclofenac with improved effect (Diclo Duo spray)].</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>TJR-candidate cohort with embedded NSAID randomisation (2011)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>NSAID randomisation incompletely described</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>S24478</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20characteristics%20and%20medication%20use%20of%20patients%20with%20knee%20osteoarthritis%20selected%20for%20total%20joint%20replacement%20surgery</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Clinical characteristics and medication use of patients with knee osteoarthritis selected for total joint replacement surgery</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="47.7" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="30.6" customWidth="1" min="4" max="4"/>
+    <col width="54.9" customWidth="1" min="4" max="4"/>
     <col width="55.8" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="20.7" customWidth="1" min="7" max="7"/>
@@ -458,7 +3609,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Group</t>
+          <t>Batch</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -540,7 +3691,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -618,7 +3769,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -696,7 +3847,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -774,7 +3925,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -856,7 +4007,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -938,7 +4089,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1016,7 +4167,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1094,7 +4245,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1176,7 +4327,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1254,7 +4405,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1 Primary: head-to-head RCT (used by reference MAs)</t>
+          <t>BATCH 1 - Head-to-head RCTs used by the reference MAs</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1332,7 +4483,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1414,7 +4565,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1496,7 +4647,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1574,7 +4725,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1652,7 +4803,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1730,7 +4881,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1808,7 +4959,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1886,7 +5037,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2 Primary: head-to-head RCT (not in any reference MA)</t>
+          <t>BATCH 2 - Head-to-head RCTs found only by your search</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1964,7 +5115,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2038,7 +5189,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2112,7 +5263,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2186,7 +5337,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2264,7 +5415,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2342,7 +5493,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>3 Exploratory combination node</t>
+          <t>BATCH 3 - Combination-node trials (topical + oral)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2424,7 +5575,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2502,7 +5653,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2584,7 +5735,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2662,7 +5813,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2740,7 +5891,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2818,7 +5969,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2896,7 +6047,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>4 NRSI safety</t>
+          <t>BATCH 4 - Non-randomised safety studies (NRSI)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2967,10 +6118,14 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3025,10 +6180,14 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3083,10 +6242,14 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3141,10 +6304,14 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3199,10 +6366,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3257,10 +6428,14 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3315,10 +6490,14 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3373,10 +6552,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3431,10 +6614,14 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3489,10 +6676,14 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>5 Retrieve only to confirm eligibility</t>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3550,7 +6741,7 @@
       <c r="A43" s="2" t="inlineStr"/>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3612,7 +6803,7 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3674,7 +6865,7 @@
       <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3736,7 +6927,7 @@
       <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3798,7 +6989,7 @@
       <c r="A47" s="2" t="inlineStr"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3860,7 +7051,7 @@
       <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3922,7 +7113,7 @@
       <c r="A49" s="2" t="inlineStr"/>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3984,7 +7175,7 @@
       <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>6 Registry only (no PDF)</t>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4046,7 +7237,7 @@
       <c r="A51" s="2" t="inlineStr"/>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>7 Excluded / not counted (report with reasons)</t>
+          <t>NO DOWNLOAD - excluded / not counted (list with reasons)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4120,7 +7311,7 @@
       <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>7 Excluded / not counted (report with reasons)</t>
+          <t>NO DOWNLOAD - excluded / not counted (list with reasons)</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4191,6 +7382,848 @@
       <c r="P52" s="2" t="inlineStr">
         <is>
           <t>Same patients as Tugwell 2004 and Simon 2009: never count as separate studies (Zeng 2021 also excluded pooled analyses). Download S05544 only if you pre-specify an age &gt;=65 subgroup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Roth 1995 (diclofenac/hyaluronan gel)</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Controlled trial, placebo gel</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac 3%/hyaluronan gel vs placebo gel in patients with uncontrolled pain on CHRONIC ORAL NSAIDs</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2 wk</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>OA, joint not stated</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>S00576</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>S14701 (RSM Round Table report)</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/8867642/</t>
+        </is>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>A controlled clinical investigation of 3% diclofenac/2.5% sodium hyaluronate topical gel in the treatment of uncontrolled pain in chronic oral NSAID users with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>Was Unclear/ANCHORED. If patients kept taking their oral NSAID and it is knee OA, this is topical+oral vs oral -&gt; combination node.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Togo 2022</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective claims cohort (Japan, MDV database)</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Oral vs non-oral NSAID users (main comparison is age &gt;=65 vs &lt;65)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>288,715</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2009-2018</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>OA and/or chronic low back pain (only 23.7% OA alone)</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>S20244</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/34538031/</t>
+        </is>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>Safety risk associated with use of nonsteroidal anti-inflammatory drugs in Japanese elderly compared with younger patients with osteoarthritis and/or chronic low back pain: A retrospective database study</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>WRONGLY REASONED EXCLUSION at T/A ("no placebo" does not apply to cohorts). Same database/group as Kikuchi 2021. Include only if it reports outcomes by route in OA patients. PMID 34538031.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac potassium 1% gel (2002, Chinese)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac potassium gel; comparator unknown (abstract = keywords only)</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>S01109</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Effect%20and%20safety%20of%201%25%20diclofenac%20potassium%20gel%20for%20external%20application%20in%20treatment%20of%20patients%20with%20osteoarthritis</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>Effect and safety of 1% diclofenac potassium gel for external application in treatment of patients with osteoarthritis</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Transdermal diclofenac multicentre trial (1987)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Transdermal diclofenac; comparator unknown</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>S21573</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Transdermic%20application%20of%20diclofenac%20-%20Results%20of%20a%20multicenter%20trial</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Transdermic application of diclofenac - Results of a multicenter trial</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Piroxicam gel in gonarthrosis (1993)</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Topical piroxicam gel; comparator unknown</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>S22576</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Efficacy%20and%20tolerance%20of%20piroxicam%20gel.%20Percutaneous%20nonsteroidal%20antirheumatic%20agents%20in%20the%20treatment%20of%20gonarthrosis</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and tolerance of piroxicam gel. Percutaneous nonsteroidal antirheumatic agents in the treatment of gonarthrosis</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Ketorolac gel 1% long-term (1993)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Topical ketorolac, knee OA; comparator unknown</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>S10571</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Long-term%20efficacy%20of%20ketorolac%20Gel%201%25%20in%20patients%20suffering%20from%20osteoarthritis%20of%20the%20knee</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>Long-term efficacy of ketorolac Gel 1% in patients suffering from osteoarthritis of the knee</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Diclo Duo spray (2010)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac spray; comparator unknown</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>S05441</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/21875024/</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>[Topical treatment with diclofenac with improved effect (Diclo Duo spray)].</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>BATCH 5 - Retrieve only to decide eligibility (most will be excluded)</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>CHECK (low probability)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>TJR-candidate cohort with embedded NSAID randomisation (2011)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Unclear at T/A, no abstract</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>NSAID randomisation incompletely described</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>S24478</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Clinical%20characteristics%20and%20medication%20use%20of%20patients%20with%20knee%20osteoarthritis%20selected%20for%20total%20joint%20replacement%20surgery</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Clinical characteristics and medication use of patients with knee osteoarthritis selected for total joint replacement surgery</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Old/no-abstract Unclear record. Only retrieve to rule out a topical-vs-oral or topical+oral design; expect exclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>NO (registry)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>IRCT20170929036477N2</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Registry record</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac gel + oral celecoxib vs placebo gel + oral celecoxib (3rd arm herbal gel)</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Knee OA / OA</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>S03348</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>https://trialsearch.who.int/Trial2.aspx?TrialID=IRCT20170929036477N2</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Comparison the effect of Stachys lavandulifolia gel vs diclofenac gel on the pain of knee</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Combination design (like Dehghan 2019). Registry only: search for a publication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NO (registry)</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>X0002 spray phase 2 (NCT03691818)</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Registry record</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>X0002 spray vs oral ibuprofen vs placebo</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Knee OA / OA</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>S21372</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT03691818</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>A Phase 2, Multicenter, Double-blind and Placebo and Active Control Study to Evaluate the Initial Efficacy and Safety of X0002 Spray in Treatment of Subjects With Osteoarthritis of the Knee</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>X0002 = "brothamine hydrochloride" (unidentified). If it is an NSAID, this is topical-vs-oral; otherwise stays ANCHORED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr"/>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>NO (registry)</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>X0002 spray phase 3 (NCT05324163)</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Registry record</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>X0002 spray vs oral celecoxib vs placebo</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Knee OA / OA</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>S06285</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT05324163</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>A Phase 3, Multicenter, Double-blind and Placebo and Active Control Study to Evaluate the Efficacy and Safety of X0002 Spray in Treatment of Subjects With Osteoarthritis of the Knee</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr"/>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>NO (registry)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Diclofenac sodium gel in knee OA (registry, 2007)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Registry record</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Topical diclofenac gel, knee OA; comparator not stated</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Knee OA / OA</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>S07217</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/scholar?q=Efficacy%20and%20safety%20of%20diclofenac%20sodium%20gel%20in%20knee%20osteoarthritis</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>Efficacy and safety of diclofenac sodium gel in knee osteoarthritis</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>No trial ID in the record; search ClinicalTrials.gov by title to see the comparator and any results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>NO DOWNLOAD - registry records (check registry for results)</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>NO (registry)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>ORCA study (NCT04099459)</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Registry record</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Observational: OA and NSAID-associated risks</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Knee OA / OA</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>S02379</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT04099459</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>ORCA Study: Osteoarthritis and Risks Associated With the Consumption of NSAIDs</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Registry only, no design detail; check whether it compares topical vs oral users.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +8232,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13795,11 +17828,19 @@
           <t>A Phase 3, Multicenter, Double-blind and Placebo and Active Control Study to Evaluate the Efficacy and Safety of X0002 Spray in Treatment of Subjects With Osteoarthritis of the Knee</t>
         </is>
       </c>
-      <c r="G264" s="2" t="inlineStr"/>
-      <c r="H264" s="2" t="inlineStr"/>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>X0002 spray phase 3 (NCT05324163)</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>main record</t>
+        </is>
+      </c>
       <c r="I264" s="2" t="inlineStr">
         <is>
-          <t>Set aside: ANCHORED stream (placebo/vehicle-only) - protocol amendment</t>
+          <t>Registry: check for results, no PDF</t>
         </is>
       </c>
     </row>
@@ -15391,7 +19432,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>